<commit_message>
27 agosto 2020 v1
</commit_message>
<xml_diff>
--- a/_downloads/ed903bb18b14ac252bb7e5c2bd096535/Valoración de FWD.xlsx
+++ b/_downloads/ed903bb18b14ac252bb7e5c2bd096535/Valoración de FWD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\DERIVADOS FINANCIEROS\CLASES\Forward\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Forward\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63E1BCA-3AFC-4FB6-8692-5099DB482EED}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4A4303-3970-4349-B915-EC67D4F93CE1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{08DF20C0-179F-4978-9BFF-8FB8AC424C27}"/>
   </bookViews>
@@ -6725,7 +6725,7 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>361358</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>73902</xdr:rowOff>
+      <xdr:rowOff>89226</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
       <mc:Choice Requires="a14">
@@ -6743,7 +6743,7 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="4544786" y="3254829"/>
-              <a:ext cx="1825486" cy="384144"/>
+              <a:ext cx="1825486" cy="399468"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -6975,13 +6975,14 @@
                     <m:sSup>
                       <m:sSupPr>
                         <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1400" i="1">
+                          <a:rPr lang="es-MX" sz="1800" i="1" kern="1200">
                             <a:solidFill>
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
+                            <a:effectLst/>
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
                           </a:rPr>
                         </m:ctrlPr>
                       </m:sSupPr>
@@ -6990,43 +6991,16 @@
                           <m:rPr>
                             <m:nor/>
                           </m:rPr>
-                          <a:rPr lang="es-MX" sz="1400">
+                          <a:rPr lang="es-MX" sz="1800" kern="1200">
                             <a:solidFill>
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>(1+</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1400">
-                            <a:solidFill>
-                              <a:schemeClr val="tx1"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>r</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1400">
-                            <a:solidFill>
-                              <a:schemeClr val="tx1"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>)</m:t>
+                            <a:effectLst/>
+                            <a:latin typeface="+mn-lt"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
+                          </a:rPr>
+                          <m:t>e</m:t>
                         </m:r>
                       </m:e>
                       <m:sup>
@@ -7034,15 +7008,16 @@
                           <m:rPr>
                             <m:nor/>
                           </m:rPr>
-                          <a:rPr lang="es-MX" sz="1400">
+                          <a:rPr lang="es-MX" sz="1800" kern="1200">
                             <a:solidFill>
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>T</m:t>
+                            <a:effectLst/>
+                            <a:latin typeface="+mn-lt"/>
+                            <a:ea typeface="+mn-ea"/>
+                            <a:cs typeface="+mn-cs"/>
+                          </a:rPr>
+                          <m:t>rT</m:t>
                         </m:r>
                       </m:sup>
                     </m:sSup>
@@ -7073,7 +7048,7 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="4544786" y="3254829"/>
-              <a:ext cx="1825486" cy="384144"/>
+              <a:ext cx="1825486" cy="399468"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -7236,51 +7211,19 @@
                   <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                   <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                 </a:rPr>
-                <a:t>" −"I)" 〖"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1400" i="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>(1+r)</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1400" i="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" 〗^"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1400" i="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>T</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1400" i="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
+                <a:t>" −"I)</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1800" i="0" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:effectLst/>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:rPr>
+                <a:t>" "e" ^"rT" </a:t>
               </a:r>
               <a:endParaRPr lang="es-CO" sz="1400">
                 <a:solidFill>
@@ -10905,8 +10848,8 @@
         <v>16</v>
       </c>
       <c r="C20" s="17">
-        <f>+(C4-C18)*EXP(C12*C8)</f>
-        <v>1862.4964108561524</v>
+        <f>+(C4-C18)*EXP(C16*C8)</f>
+        <v>1860.8584110574132</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>11</v>
@@ -10917,8 +10860,8 @@
         <v>16</v>
       </c>
       <c r="C21" s="18">
-        <f>+(C4-C18)*(1+C11)^C8</f>
-        <v>1862.4964108561524</v>
+        <f>+(C4-C18)*(1+C15)^C8</f>
+        <v>1860.8584110574132</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>11</v>
@@ -11048,7 +10991,7 @@
       </c>
       <c r="C36" s="19">
         <f>+(C33-C20)*EXP(-C31*C28)</f>
-        <v>240.72641462059886</v>
+        <v>242.36158005818089</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>18</v>
@@ -11060,7 +11003,7 @@
       </c>
       <c r="C37" s="20">
         <f>+C36*C9</f>
-        <v>1203632.0731029944</v>
+        <v>1211807.9002909046</v>
       </c>
       <c r="D37" s="6" t="s">
         <v>19</v>
@@ -11077,7 +11020,7 @@
       </c>
       <c r="C39" s="11">
         <f>-C36</f>
-        <v>-240.72641462059886</v>
+        <v>-242.36158005818089</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>18</v>
@@ -11089,7 +11032,7 @@
       </c>
       <c r="C40" s="11">
         <f>-C37</f>
-        <v>-1203632.0731029944</v>
+        <v>-1211807.9002909046</v>
       </c>
       <c r="D40" s="6" t="s">
         <v>19</v>

</xml_diff>